<commit_message>
Deploying to gh-pages from @ NIH-NCPI/ncpi-fhir-ig-2@168df1bedc3b701e0e1f6a6258c635387b77916f 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-SharedDataModelAliquot.xlsx
+++ b/StructureDefinition-SharedDataModelAliquot.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-13T18:03:13+00:00</t>
+    <t>2026-02-06T18:07:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -260,7 +260,7 @@
     <t>SharedDataModelAliquot.sample</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {valueset-reference}
+    <t xml:space="preserve">Reference(https://nih-ncpi.github.io/ncpi-fhir-ig-2/StructureDefinition/ncpi-sample)
 </t>
   </si>
   <si>
@@ -605,7 +605,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="25.94921875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="65.69140625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>